<commit_message>
feat: expand financial analysis dashboard
</commit_message>
<xml_diff>
--- a/sektorler/Elektrik - Doğalgaz Dağıtım.xlsx
+++ b/sektorler/Elektrik - Doğalgaz Dağıtım.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:X8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,53 +553,53 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>ARASE</t>
+          <t>ENJSA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19952112656</v>
+        <v>100728570000</v>
       </c>
       <c r="C2" t="n">
-        <v>250000000</v>
+        <v>1181069000</v>
       </c>
       <c r="D2" t="n">
-        <v>2459876674</v>
+        <v>69429507000</v>
       </c>
       <c r="E2" t="n">
-        <v>104.5</v>
+        <v>109.8000030517578</v>
       </c>
       <c r="F2" t="n">
-        <v>26125000000</v>
+        <v>129681379804.3365</v>
       </c>
       <c r="G2" t="n">
-        <v>28584876674</v>
+        <v>199110886804.3365</v>
       </c>
       <c r="H2" t="n">
-        <v>32719668747</v>
+        <v>251859885346</v>
       </c>
       <c r="I2" t="n">
-        <v>7553214745</v>
+        <v>41134966606</v>
       </c>
       <c r="J2" t="n">
-        <v>7896182616</v>
+        <v>48257752503</v>
       </c>
       <c r="K2" t="n">
-        <v>2239980382</v>
+        <v>5539063054</v>
       </c>
       <c r="L2" t="n">
-        <v>11.66304857396738</v>
+        <v>23.41215085296564</v>
       </c>
       <c r="M2" t="n">
-        <v>3.620088093717411</v>
+        <v>4.125987566287066</v>
       </c>
       <c r="N2" t="n">
-        <v>0.8736297697580111</v>
+        <v>0.7905621275527941</v>
       </c>
       <c r="O2" t="n">
-        <v>1.30938514885258</v>
+        <v>1.287433940582464</v>
       </c>
       <c r="P2" t="n">
-        <v>28.91182677511961</v>
+        <v>31.72002539459751</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -607,77 +607,77 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>53260667141.3076</v>
+        <v>93779925679.7412</v>
       </c>
       <c r="S2" t="n">
-        <v>33848941916.4251</v>
+        <v>142850047044.8416</v>
       </c>
       <c r="T2" t="n">
-        <v>24974405233.94387</v>
+        <v>150696662909.4548</v>
       </c>
       <c r="U2" t="n">
-        <v>27664850278.55286</v>
+        <v>130951223094.5845</v>
       </c>
       <c r="V2" t="n">
-        <v>34937216142.55736</v>
+        <v>129569464682.1555</v>
       </c>
       <c r="W2" t="n">
-        <v>139.7488645702294</v>
+        <v>109.7052455717283</v>
       </c>
       <c r="X2" t="n">
-        <v>-25.22300605348781</v>
+        <v>0.08637461183895745</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ENJSA</t>
+          <t>ARASE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95768408000</v>
+        <v>22394326381</v>
       </c>
       <c r="C3" t="n">
-        <v>1181069000</v>
+        <v>250000000</v>
       </c>
       <c r="D3" t="n">
-        <v>63562449000</v>
+        <v>1001576225</v>
       </c>
       <c r="E3" t="n">
-        <v>122.8000030517578</v>
+        <v>112.1999969482422</v>
       </c>
       <c r="F3" t="n">
-        <v>145035276804.3365</v>
+        <v>28049999237.06055</v>
       </c>
       <c r="G3" t="n">
-        <v>208597725804.3365</v>
+        <v>29051575462.06055</v>
       </c>
       <c r="H3" t="n">
-        <v>233065038000</v>
+        <v>38416180991</v>
       </c>
       <c r="I3" t="n">
-        <v>36912096000</v>
+        <v>8742876923</v>
       </c>
       <c r="J3" t="n">
-        <v>43277287000</v>
+        <v>9118281875</v>
       </c>
       <c r="K3" t="n">
-        <v>3171282000</v>
+        <v>2698381907</v>
       </c>
       <c r="L3" t="n">
-        <v>45.73395768788034</v>
+        <v>10.39511833528631</v>
       </c>
       <c r="M3" t="n">
-        <v>4.820027785113622</v>
+        <v>3.186079994051571</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8950193799738275</v>
+        <v>0.7562327829740974</v>
       </c>
       <c r="O3" t="n">
-        <v>1.514437587856076</v>
+        <v>1.252549362719791</v>
       </c>
       <c r="P3" t="n">
-        <v>25.45042613997778</v>
+        <v>31.16890253404583</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -685,25 +685,25 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>75404497454.75507</v>
+        <v>45685353682.92602</v>
       </c>
       <c r="S3" t="n">
-        <v>135438414985.1805</v>
+        <v>39108555508.95987</v>
       </c>
       <c r="T3" t="n">
-        <v>131854320186.0848</v>
+        <v>32574262072.86945</v>
       </c>
       <c r="U3" t="n">
-        <v>132788878772.6262</v>
+        <v>29113531840.78032</v>
       </c>
       <c r="V3" t="n">
-        <v>118871527849.6616</v>
+        <v>36620425776.38391</v>
       </c>
       <c r="W3" t="n">
-        <v>100.6474031996959</v>
+        <v>146.4817031055356</v>
       </c>
       <c r="X3" t="n">
-        <v>22.01010572335247</v>
+        <v>-23.40340495126174</v>
       </c>
     </row>
     <row r="4">
@@ -722,13 +722,13 @@
         <v>-4762675109</v>
       </c>
       <c r="E4" t="n">
-        <v>51.09999847412109</v>
+        <v>44.06000137329102</v>
       </c>
       <c r="F4" t="n">
-        <v>35769998931.88477</v>
+        <v>30842000961.30371</v>
       </c>
       <c r="G4" t="n">
-        <v>31007323822.88477</v>
+        <v>26079325852.30371</v>
       </c>
       <c r="H4" t="n">
         <v>54073694479</v>
@@ -743,19 +743,19 @@
         <v>3291590642</v>
       </c>
       <c r="L4" t="n">
-        <v>10.86708610586844</v>
+        <v>9.369938220070962</v>
       </c>
       <c r="M4" t="n">
-        <v>4.336348631338439</v>
+        <v>3.647172184605034</v>
       </c>
       <c r="N4" t="n">
-        <v>0.5734271371993407</v>
+        <v>0.482292288396012</v>
       </c>
       <c r="O4" t="n">
-        <v>1.06714764803664</v>
+        <v>0.9201277542466176</v>
       </c>
       <c r="P4" t="n">
-        <v>10.25804470385166</v>
+        <v>11.89709605937609</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -763,150 +763,306 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>78265111140.15865</v>
+        <v>55728761843.93253</v>
       </c>
       <c r="S4" t="n">
-        <v>37642918834.61572</v>
+        <v>36217057960.21206</v>
       </c>
       <c r="T4" t="n">
-        <v>50101550316.19264</v>
+        <v>52023219368.21839</v>
       </c>
       <c r="U4" t="n">
-        <v>46476546685.04227</v>
+        <v>43576395731.94686</v>
       </c>
       <c r="V4" t="n">
-        <v>53121531744.00232</v>
+        <v>46886358726.07746</v>
       </c>
       <c r="W4" t="n">
-        <v>75.88790249143189</v>
+        <v>66.98051246582494</v>
       </c>
       <c r="X4" t="n">
-        <v>-32.66384127576786</v>
+        <v>-34.21967113827103</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>SEKTÖR TOPLAM</t>
+          <t>AHGAZ</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>149239780149</v>
+        <v>54701388025</v>
       </c>
       <c r="C5" t="n">
-        <v>2131069000</v>
+        <v>2600000000</v>
       </c>
       <c r="D5" t="n">
-        <v>61259650565</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>-36723863292</v>
+      </c>
+      <c r="E5" t="n">
+        <v>32.22000122070312</v>
+      </c>
       <c r="F5" t="n">
-        <v>206930275736.2213</v>
+        <v>83772003173.82812</v>
       </c>
       <c r="G5" t="n">
-        <v>268189926301.2213</v>
+        <v>47048139881.82812</v>
       </c>
       <c r="H5" t="n">
-        <v>319858401226</v>
+        <v>46379576614</v>
       </c>
       <c r="I5" t="n">
-        <v>48134613226</v>
+        <v>9394355260</v>
       </c>
       <c r="J5" t="n">
-        <v>58324030251</v>
+        <v>13279599252</v>
       </c>
       <c r="K5" t="n">
-        <v>8702853024</v>
+        <v>3814522180</v>
       </c>
       <c r="L5" t="n">
-        <v>23.77729178759727</v>
+        <v>21.96133597362596</v>
       </c>
       <c r="M5" t="n">
-        <v>4.598274933111692</v>
+        <v>3.542888530671763</v>
       </c>
       <c r="N5" t="n">
-        <v>0.8384645370365881</v>
+        <v>1.014415036027438</v>
       </c>
       <c r="O5" t="n">
-        <v>1.386562453587264</v>
+        <v>1.531442001719263</v>
       </c>
       <c r="P5" t="n">
-        <v>0.2326127148613008</v>
+        <v>11.21419436575556</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>Elektrik - Doğalgaz Dağıtım</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>64582331534.53544</v>
+      </c>
+      <c r="S5" t="n">
+        <v>95139086979.29306</v>
+      </c>
+      <c r="T5" t="n">
+        <v>77259729287.63695</v>
+      </c>
+      <c r="U5" t="n">
+        <v>71114021243.87555</v>
+      </c>
+      <c r="V5" t="n">
+        <v>77023792261.33525</v>
+      </c>
+      <c r="W5" t="n">
+        <v>29.62453548512894</v>
+      </c>
+      <c r="X5" t="n">
+        <v>8.761203148238629</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
+          <t>ENERY</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>59206007042</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9000000000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-5422576706</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8.819999694824219</v>
+      </c>
+      <c r="F6" t="n">
+        <v>79379997253.41797</v>
+      </c>
+      <c r="G6" t="n">
+        <v>73957420547.41797</v>
+      </c>
+      <c r="H6" t="n">
+        <v>38614225948</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4392619737</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7499212349</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5430920825</v>
+      </c>
+      <c r="L6" t="n">
+        <v>14.61630537643089</v>
+      </c>
+      <c r="M6" t="n">
+        <v>9.862025117515174</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1.915289475102078</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1.340742286455947</v>
+      </c>
+      <c r="P6" t="n">
+        <v>5.533660731905432</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Elektrik - Doğalgaz Dağıtım</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>91949007688.81169</v>
+      </c>
+      <c r="S6" t="n">
+        <v>38410632936.64034</v>
+      </c>
+      <c r="T6" t="n">
+        <v>39171506791.76732</v>
+      </c>
+      <c r="U6" t="n">
+        <v>76970208518.75967</v>
+      </c>
+      <c r="V6" t="n">
+        <v>61625338983.99476</v>
+      </c>
+      <c r="W6" t="n">
+        <v>6.847259887110528</v>
+      </c>
+      <c r="X6" t="n">
+        <v>28.81064601370296</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>SEKTÖR TOPLAM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>270549550941</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13731069000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>23521968118</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>351725380429.9469</v>
+      </c>
+      <c r="G7" t="n">
+        <v>375247348547.9469</v>
+      </c>
+      <c r="H7" t="n">
+        <v>429343563378</v>
+      </c>
+      <c r="I7" t="n">
+        <v>67334121007</v>
+      </c>
+      <c r="J7" t="n">
+        <v>85305406614</v>
+      </c>
+      <c r="K7" t="n">
+        <v>20774478608</v>
+      </c>
+      <c r="L7" t="n">
+        <v>16.93064779466964</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4.398869467276682</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.8740025018555454</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1.300040525687841</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.1914394716829681</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Elektrik - Doğalgaz Dağıtım</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
           <t>SEKTÖR Median</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>33519259493</v>
-      </c>
-      <c r="C6" t="n">
-        <v>700000000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2459876674</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="n">
-        <v>35769998931.88477</v>
-      </c>
-      <c r="G6" t="n">
-        <v>31007323822.88477</v>
-      </c>
-      <c r="H6" t="n">
-        <v>54073694479</v>
-      </c>
-      <c r="I6" t="n">
-        <v>7553214745</v>
-      </c>
-      <c r="J6" t="n">
-        <v>7896182616</v>
-      </c>
-      <c r="K6" t="n">
-        <v>3171282000</v>
-      </c>
-      <c r="L6" t="n">
-        <v>11.66304857396738</v>
-      </c>
-      <c r="M6" t="n">
-        <v>4.336348631338439</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.8736297697580111</v>
-      </c>
-      <c r="O6" t="n">
-        <v>1.30938514885258</v>
-      </c>
-      <c r="P6" t="n">
-        <v>25.45042613997778</v>
-      </c>
-      <c r="Q6" t="inlineStr">
+      <c r="B8" t="n">
+        <v>54701388025</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1181069000</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-4762675109</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>79379997253.41797</v>
+      </c>
+      <c r="G8" t="n">
+        <v>47048139881.82812</v>
+      </c>
+      <c r="H8" t="n">
+        <v>46379576614</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8742876923</v>
+      </c>
+      <c r="J8" t="n">
+        <v>9118281875</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3814522180</v>
+      </c>
+      <c r="L8" t="n">
+        <v>14.61630537643089</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3.647172184605034</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.7905621275527941</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1.287433940582464</v>
+      </c>
+      <c r="P8" t="n">
+        <v>11.89709605937609</v>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Elektrik - Doğalgaz Dağıtım</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>